<commit_message>
Add local data and correct errors with PO tables
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/NarayenLongTermGrazingTrial/Observed.xlsx
+++ b/Tests/Validation/System/NarayenLongTermGrazingTrial/Observed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Repos\ApsimX\Tests\Validation\System\NarayenLongTermGrazingTrial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4822A1D4-7FC3-4113-9F95-F6889E8F698D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2263B1-FA8F-4BE2-98FA-8AE4FA18F607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,6 +401,9 @@
     <col min="5" max="5" width="20.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>